<commit_message>
Añadidas soluciones en excel.
</commit_message>
<xml_diff>
--- a/soluciones.xlsx
+++ b/soluciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ceu365-my.sharepoint.com/personal/asalber_ceu_es/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{35A37B39-1725-4E39-8AE6-523674FB9691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{11509F91-E2A6-4148-87A9-E83BB5155C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" firstSheet="1" activeTab="16" xr2:uid="{4F73E1E8-AEEB-46FA-85F6-1B58A425B0CB}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" firstSheet="17" activeTab="19" xr2:uid="{4F73E1E8-AEEB-46FA-85F6-1B58A425B0CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Ej.1.4" sheetId="9" r:id="rId1"/>
@@ -30,7 +30,10 @@
     <sheet name="Ej.2.4" sheetId="18" r:id="rId15"/>
     <sheet name="Ej.2.5" sheetId="5" r:id="rId16"/>
     <sheet name="Ej.2.6" sheetId="19" r:id="rId17"/>
-    <sheet name="Ej.2.11" sheetId="7" r:id="rId18"/>
+    <sheet name="Ej.2.7" sheetId="20" r:id="rId18"/>
+    <sheet name="Ej.2.10" sheetId="21" r:id="rId19"/>
+    <sheet name="Ej.2.11" sheetId="22" r:id="rId20"/>
+    <sheet name="Ej.2.12" sheetId="7" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -53,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="94">
   <si>
     <t>n</t>
   </si>
@@ -187,7 +190,7 @@
     <t xml:space="preserve">Decisión </t>
   </si>
   <si>
-    <t>Rechazar h0</t>
+    <t>Rechazar H0</t>
   </si>
   <si>
     <t>Media = 20</t>
@@ -220,9 +223,6 @@
     <t>Decisión</t>
   </si>
   <si>
-    <t>Rechazar H0</t>
-  </si>
-  <si>
     <t>Helado</t>
   </si>
   <si>
@@ -242,6 +242,90 @@
   </si>
   <si>
     <t>Cuasivarianza muestral</t>
+  </si>
+  <si>
+    <t>Media = 46,5</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>Media &gt; 46,5</t>
+  </si>
+  <si>
+    <t>Media = 48,5</t>
+  </si>
+  <si>
+    <t>Cuasivarianza</t>
+  </si>
+  <si>
+    <t>Alfa</t>
+  </si>
+  <si>
+    <t>Beta</t>
+  </si>
+  <si>
+    <t>Z alfa</t>
+  </si>
+  <si>
+    <t>Z beta</t>
+  </si>
+  <si>
+    <t>Frontera región aceptación</t>
+  </si>
+  <si>
+    <t>Estadístico con hipótesis alternativa</t>
+  </si>
+  <si>
+    <t>Error beta</t>
+  </si>
+  <si>
+    <t>Potencia</t>
+  </si>
+  <si>
+    <t>Sin aditivo</t>
+  </si>
+  <si>
+    <t>Con Aditivo</t>
+  </si>
+  <si>
+    <t>Diferencia</t>
+  </si>
+  <si>
+    <t>Media = 0</t>
+  </si>
+  <si>
+    <t>Media &gt; 0</t>
+  </si>
+  <si>
+    <t>p1 = p2</t>
+  </si>
+  <si>
+    <t>p1 != p2</t>
+  </si>
+  <si>
+    <t>frecuencia 1</t>
+  </si>
+  <si>
+    <t>frecuencia 2</t>
+  </si>
+  <si>
+    <t>p1</t>
+  </si>
+  <si>
+    <t>p2</t>
+  </si>
+  <si>
+    <t>Varianza 1 = Varianza 2</t>
+  </si>
+  <si>
+    <t>Media1 = Media 2</t>
+  </si>
+  <si>
+    <t>Varianza 1 != Varianza 2</t>
+  </si>
+  <si>
+    <t>Media 1 != Media 2</t>
   </si>
   <si>
     <t>Estadístico medias</t>
@@ -1543,7 +1627,7 @@
         <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1561,7 +1645,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C1" t="s">
         <v>32</v>
@@ -1578,7 +1662,7 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15">
@@ -1670,7 +1754,7 @@
         <v>54</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15">
@@ -1758,7 +1842,7 @@
         <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1766,7 +1850,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1779,7 +1863,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B4">
         <v>9</v>
@@ -1787,7 +1871,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5">
         <f>3.5^2</f>
@@ -1825,7 +1909,7 @@
         <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1834,104 +1918,140 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05F25D3-2972-4151-B9E8-34D8906E9CEF}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.85"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C228AD1-3AA1-4975-ACC4-5BCDB558DDEC}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
-    <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1">
-        <v>100</v>
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
+        <v>62</v>
       </c>
       <c r="D1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1">
-        <v>1630</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>32</v>
+      </c>
+      <c r="E1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2">
-        <v>120</v>
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>64</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2">
-        <v>1780</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15">
+        <v>34</v>
+      </c>
+      <c r="E2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2">
+        <f>E6^2</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B3">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <f>((B1-1)*B5+(B2-1)*B6)/(B1+B2-2)</f>
-        <v>24192.201834862386</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15">
+        <v>40</v>
+      </c>
+      <c r="G3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H3">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="B4">
-        <v>160</v>
+        <v>46.5</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E4">
-        <f>SQRT(E3)</f>
-        <v>155.53842558950629</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15">
+        <v>48.5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B5">
-        <f>B3^2</f>
-        <v>22500</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="E5">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15">
+        <v>49</v>
+      </c>
+      <c r="G5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H5">
+        <f>-_xlfn.NORM.INV(H3,0,1)</f>
+        <v>1.6448536269514726</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B6">
-        <f>B4^2</f>
-        <v>25600</v>
+        <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E6">
-        <f>1-E5</f>
-        <v>5.0000000000000044E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s">
+        <v>70</v>
+      </c>
+      <c r="H6">
+        <f>-_xlfn.NORM.INV(H4,0,1)</f>
+        <v>0.84162123357291452</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1939,41 +2059,293 @@
         <v>0.05</v>
       </c>
       <c r="D7" t="s">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="E7">
-        <f>(E1-E2)/(E4*SQRT((B1+B2)/(B1*B2)))</f>
-        <v>-7.1225063171060929</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="15">
+        <v>0.05</v>
+      </c>
+      <c r="G7" t="s">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f>(H5+H6)^2*H2/H1^2</f>
+        <v>75.736326092242194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="B8">
-        <f>B5/B6</f>
-        <v>0.87890625</v>
+        <f>(B5-B4)/(B6/SQRT(B3))</f>
+        <v>2.2587697572631282</v>
       </c>
       <c r="D8" t="s">
-        <v>65</v>
+        <v>6</v>
       </c>
       <c r="E8">
-        <f>_xlfn.T.DIST.2T(ABS(E7),B1+B2-2)</f>
-        <v>1.5219901875321142E-11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="15">
+        <f>_xlfn.T.INV(1-E7,E3-1)</f>
+        <v>1.6848751217112248</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="B9">
-        <f>2*_xlfn.F.DIST(B8,B1-1,B2-1,TRUE)</f>
-        <v>0.5079833817134547</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="15"/>
-    <row r="11" spans="1:5" ht="15"/>
-    <row r="12" spans="1:5" ht="15"/>
+        <f>_xlfn.T.DIST.RT(B8,B3-1)</f>
+        <v>1.4782679871508761E-2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9">
+        <f>B4+E8*E6/SQRT(E3)</f>
+        <v>48.364815035146307</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10">
+        <f>(E9-E4)/(E6/SQRT(E3))</f>
+        <v>-0.12214068409927997</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="D11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11">
+        <f>_xlfn.T.DIST(E10,E3-1,TRUE)</f>
+        <v>0.45170740733104819</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="D12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12">
+        <f>1-E11</f>
+        <v>0.54829259266895181</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A8413D7-C758-4B5D-807C-C3DC412C9661}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>0.38</v>
+      </c>
+      <c r="B2">
+        <v>0.38</v>
+      </c>
+      <c r="C2">
+        <f>A2-B2</f>
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>0.42</v>
+      </c>
+      <c r="B3">
+        <v>0.36</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C11" si="0">A3-B3</f>
+        <v>0.06</v>
+      </c>
+      <c r="E3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <f>COUNT(C2:C11)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>0.41</v>
+      </c>
+      <c r="B4">
+        <v>0.38</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>2.9999999999999971E-2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>0.39</v>
+      </c>
+      <c r="B5">
+        <v>0.32</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5">
+        <f>AVERAGE(C2:C11)</f>
+        <v>3.4999999999999996E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>0.45</v>
+      </c>
+      <c r="B6">
+        <v>0.39</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>0.06</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <f>STDEV(C2:C11)</f>
+        <v>2.7182510717166826E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>0.47</v>
+      </c>
+      <c r="B7">
+        <v>0.45</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>1.9999999999999962E-2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>0.44</v>
+      </c>
+      <c r="B8">
+        <v>0.39</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>4.9999999999999989E-2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8">
+        <f>(F5-F4)/(F6/SQRT(F3))</f>
+        <v>4.0717253552297752</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>0.38</v>
+      </c>
+      <c r="B9">
+        <v>0.39</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>-1.0000000000000009E-2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9">
+        <f>_xlfn.T.DIST.RT(F8,F3-1)</f>
+        <v>1.3962075252613804E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10">
+        <v>0.4</v>
+      </c>
+      <c r="B10">
+        <v>0.35</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11">
+        <v>0.5</v>
+      </c>
+      <c r="B11">
+        <v>0.48</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>2.0000000000000018E-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2152,6 +2524,306 @@
         <v>4.1690268703801108</v>
       </c>
     </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27AFE8AC-1C70-4F04-8713-97CCAF2C5F4C}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7">
+        <f>B5/B3</f>
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8">
+        <f>B6/B4</f>
+        <v>0.47199999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10">
+        <f>(B7-B8)/SQRT(B7*(1-B7)/B3 + B8*(1-B8)/B4)</f>
+        <v>2.4025790617070459</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11">
+        <f>2*(1-_xlfn.NORM.S.DIST(B10,TRUE))</f>
+        <v>1.6279914989633104E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05F25D3-2972-4151-B9E8-34D8906E9CEF}">
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.85"/>
+  <cols>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>100</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>120</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4">
+        <v>1780</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5">
+        <v>150</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5">
+        <f>((B3-1)*B7+(B4-1)*B8)/(B3+B4-2)</f>
+        <v>24192.201834862386</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6">
+        <v>160</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <f>SQRT(E5)</f>
+        <v>155.53842558950629</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7">
+        <f>B5^2</f>
+        <v>22500</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8">
+        <f>B6^2</f>
+        <v>25600</v>
+      </c>
+      <c r="D8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8">
+        <f>1-E7</f>
+        <v>5.0000000000000044E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>0.05</v>
+      </c>
+      <c r="D9" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9">
+        <f>(E3-E4)/(E6*SQRT((B3+B4)/(B3*B4)))</f>
+        <v>-7.1225063171060929</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15">
+      <c r="A10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10">
+        <f>B7/B8</f>
+        <v>0.87890625</v>
+      </c>
+      <c r="D10" t="s">
+        <v>92</v>
+      </c>
+      <c r="E10">
+        <f>_xlfn.T.DIST.2T(ABS(E9),B3+B4-2)</f>
+        <v>1.5219901875321142E-11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15">
+      <c r="A11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11">
+        <f>2*_xlfn.F.DIST(B10,B3-1,B4-1,TRUE)</f>
+        <v>0.5079833817134547</v>
+      </c>
+      <c r="D11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15"/>
+    <row r="14" spans="1:5" ht="15"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3496,15 +4168,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <CultureName xmlns="5f6d3a9b-301d-40b0-aa2e-400b335c2b3f" xsi:nil="true"/>
@@ -3556,14 +4219,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B583D474-8EA0-4151-9D3B-4ECF0A63F27F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B461BA2-5B58-49A0-98FD-E5A11A7E810C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05A72ACB-C6CB-43C4-A81C-59AC4500343C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05A72ACB-C6CB-43C4-A81C-59AC4500343C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B461BA2-5B58-49A0-98FD-E5A11A7E810C}"/>
 </file>
</xml_diff>